<commit_message>
Block self-nomination server-side, colour-code dashboard flags
</commit_message>
<xml_diff>
--- a/data/Star_Awards_Mock_Nominations.xlsx
+++ b/data/Star_Awards_Mock_Nominations.xlsx
@@ -9,9 +9,12 @@
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Form Responses" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
-  <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
+</file>
+
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="0" uniqueCount="0"/>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
@@ -461,14 +464,14 @@
   <dimension ref="A1:H51"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="6" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="26" customWidth="1" min="4" max="4"/>
-    <col width="30" customWidth="1" min="5" max="5"/>
-    <col width="30" customWidth="1" min="6" max="6"/>
-    <col width="90" customWidth="1" min="7" max="7"/>
-    <col width="26" customWidth="1" min="8" max="8"/>
+    <col min="1" max="1" customWidth="true" width="6.0"/>
+    <col min="2" max="2" customWidth="true" width="18.0"/>
+    <col min="3" max="3" customWidth="true" width="18.0"/>
+    <col min="4" max="4" customWidth="true" width="26.0"/>
+    <col min="5" max="5" customWidth="true" width="30.0"/>
+    <col min="6" max="6" customWidth="true" width="30.0"/>
+    <col min="7" max="7" customWidth="true" width="90.0"/>
+    <col min="8" max="8" customWidth="true" width="26.0"/>
   </cols>
   <sheetData>
     <row r="1" ht="30" customHeight="1">
@@ -2338,9 +2341,7 @@
       </c>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n">
-        <v>49</v>
-      </c>
+      <c r="A50" s="2"/>
       <c r="B50" s="3" t="n">
         <v>46245.37430555555</v>
       </c>
@@ -2376,9 +2377,7 @@
       </c>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n">
-        <v>50</v>
-      </c>
+      <c r="A51" s="2"/>
       <c r="B51" s="3" t="n">
         <v>46246.37708333333</v>
       </c>

</xml_diff>